<commit_message>
finished project for good++
</commit_message>
<xml_diff>
--- a/results/excel_reports/independent_mobilenet_v2_black.xlsx
+++ b/results/excel_reports/independent_mobilenet_v2_black.xlsx
@@ -1136,7 +1136,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
@@ -1236,64 +1236,64 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.801</v>
+        <v>0.804</v>
       </c>
       <c r="C2" t="n">
-        <v>0.79</v>
+        <v>0.74</v>
       </c>
       <c r="D2" t="n">
-        <v>0.78</v>
+        <v>0.726</v>
       </c>
       <c r="E2" t="n">
-        <v>0.774</v>
+        <v>0.718</v>
       </c>
       <c r="F2" t="n">
-        <v>0.767</v>
+        <v>0.722</v>
       </c>
       <c r="G2" t="n">
-        <v>0.765</v>
+        <v>0.714</v>
       </c>
       <c r="H2" t="n">
-        <v>0.76</v>
+        <v>0.713</v>
       </c>
       <c r="I2" t="n">
-        <v>0.756</v>
+        <v>0.695</v>
       </c>
       <c r="J2" t="n">
-        <v>0.755</v>
+        <v>0.681</v>
       </c>
       <c r="K2" t="n">
-        <v>0.72</v>
+        <v>0.662</v>
       </c>
       <c r="L2" t="n">
-        <v>0.7</v>
+        <v>0.654</v>
       </c>
       <c r="M2" t="n">
-        <v>0.697</v>
+        <v>0.626</v>
       </c>
       <c r="N2" t="n">
-        <v>0.672</v>
+        <v>0.613</v>
       </c>
       <c r="O2" t="n">
-        <v>0.636</v>
+        <v>0.5629999999999999</v>
       </c>
       <c r="P2" t="n">
-        <v>0.601</v>
+        <v>0.512</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.451</v>
       </c>
       <c r="R2" t="n">
-        <v>0.466</v>
+        <v>0.36</v>
       </c>
       <c r="S2" t="n">
-        <v>0.354</v>
+        <v>0.247</v>
       </c>
       <c r="T2" t="n">
-        <v>0.236</v>
+        <v>0.136</v>
       </c>
       <c r="U2" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.036</v>
       </c>
       <c r="V2" t="n">
         <v>0.001</v>
@@ -1306,7 +1306,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.801</v>
+        <v>0.8008008008008008</v>
       </c>
       <c r="C3" t="n">
         <v>0.785</v>
@@ -1376,7 +1376,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.801</v>
+        <v>0.8008008008008008</v>
       </c>
       <c r="C4" t="n">
         <v>0.79</v>
@@ -1446,7 +1446,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.801</v>
+        <v>0.8008008008008008</v>
       </c>
       <c r="C5" t="n">
         <v>0.789</v>
@@ -1516,7 +1516,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.801</v>
+        <v>0.8008008008008008</v>
       </c>
       <c r="C6" t="n">
         <v>0.786</v>
@@ -1586,7 +1586,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.801</v>
+        <v>0.8008008008008008</v>
       </c>
       <c r="C7" t="n">
         <v>0.784</v>
@@ -1656,7 +1656,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.801</v>
+        <v>0.8008008008008008</v>
       </c>
       <c r="C8" t="n">
         <v>0.793</v>
@@ -1747,7 +1747,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
@@ -1843,68 +1843,68 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>u2net</t>
+          <t>dino+u2net_sum</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.945</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.926</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.912</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9379999999999999</v>
+        <v>0.905</v>
       </c>
       <c r="F2" t="n">
-        <v>0.93</v>
+        <v>0.9</v>
       </c>
       <c r="G2" t="n">
-        <v>0.93</v>
+        <v>0.898</v>
       </c>
       <c r="H2" t="n">
-        <v>0.925</v>
+        <v>0.889</v>
       </c>
       <c r="I2" t="n">
-        <v>0.92</v>
+        <v>0.882</v>
       </c>
       <c r="J2" t="n">
-        <v>0.92</v>
+        <v>0.87</v>
       </c>
       <c r="K2" t="n">
-        <v>0.914</v>
+        <v>0.864</v>
       </c>
       <c r="L2" t="n">
-        <v>0.894</v>
+        <v>0.845</v>
       </c>
       <c r="M2" t="n">
-        <v>0.888</v>
+        <v>0.833</v>
       </c>
       <c r="N2" t="n">
-        <v>0.875</v>
+        <v>0.819</v>
       </c>
       <c r="O2" t="n">
-        <v>0.842</v>
+        <v>0.78</v>
       </c>
       <c r="P2" t="n">
-        <v>0.805</v>
+        <v>0.731</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.753</v>
+        <v>0.672</v>
       </c>
       <c r="R2" t="n">
-        <v>0.694</v>
+        <v>0.582</v>
       </c>
       <c r="S2" t="n">
-        <v>0.619</v>
+        <v>0.425</v>
       </c>
       <c r="T2" t="n">
-        <v>0.472</v>
+        <v>0.261</v>
       </c>
       <c r="U2" t="n">
-        <v>0.234</v>
+        <v>0.092</v>
       </c>
       <c r="V2" t="n">
         <v>0.005</v>
@@ -1913,68 +1913,68 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>u2net+dino_320</t>
+          <t>u2net</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.9419419419419419</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="D3" t="n">
-        <v>0.9340000000000001</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="E3" t="n">
-        <v>0.929</v>
+        <v>0.9379999999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>0.928</v>
+        <v>0.93</v>
       </c>
       <c r="G3" t="n">
-        <v>0.922</v>
+        <v>0.93</v>
       </c>
       <c r="H3" t="n">
-        <v>0.915</v>
+        <v>0.925</v>
       </c>
       <c r="I3" t="n">
-        <v>0.916</v>
+        <v>0.92</v>
       </c>
       <c r="J3" t="n">
-        <v>0.915</v>
+        <v>0.92</v>
       </c>
       <c r="K3" t="n">
-        <v>0.904</v>
+        <v>0.914</v>
       </c>
       <c r="L3" t="n">
-        <v>0.895</v>
+        <v>0.894</v>
       </c>
       <c r="M3" t="n">
-        <v>0.879</v>
+        <v>0.888</v>
       </c>
       <c r="N3" t="n">
-        <v>0.876</v>
+        <v>0.875</v>
       </c>
       <c r="O3" t="n">
-        <v>0.851</v>
+        <v>0.842</v>
       </c>
       <c r="P3" t="n">
-        <v>0.819</v>
+        <v>0.805</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.784</v>
+        <v>0.753</v>
       </c>
       <c r="R3" t="n">
-        <v>0.724</v>
+        <v>0.694</v>
       </c>
       <c r="S3" t="n">
-        <v>0.611</v>
+        <v>0.619</v>
       </c>
       <c r="T3" t="n">
-        <v>0.48</v>
+        <v>0.472</v>
       </c>
       <c r="U3" t="n">
-        <v>0.242</v>
+        <v>0.234</v>
       </c>
       <c r="V3" t="n">
         <v>0.005</v>
@@ -1983,68 +1983,68 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>u2net+dino</t>
+          <t>u2net+dino_320</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.9419419419419419</v>
       </c>
       <c r="C4" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.9409999999999999</v>
       </c>
       <c r="D4" t="n">
-        <v>0.931</v>
+        <v>0.9340000000000001</v>
       </c>
       <c r="E4" t="n">
-        <v>0.93</v>
+        <v>0.929</v>
       </c>
       <c r="F4" t="n">
-        <v>0.931</v>
+        <v>0.928</v>
       </c>
       <c r="G4" t="n">
-        <v>0.925</v>
+        <v>0.922</v>
       </c>
       <c r="H4" t="n">
-        <v>0.919</v>
+        <v>0.915</v>
       </c>
       <c r="I4" t="n">
-        <v>0.917</v>
+        <v>0.916</v>
       </c>
       <c r="J4" t="n">
         <v>0.915</v>
       </c>
       <c r="K4" t="n">
-        <v>0.907</v>
+        <v>0.904</v>
       </c>
       <c r="L4" t="n">
-        <v>0.891</v>
+        <v>0.895</v>
       </c>
       <c r="M4" t="n">
-        <v>0.88</v>
+        <v>0.879</v>
       </c>
       <c r="N4" t="n">
-        <v>0.877</v>
+        <v>0.876</v>
       </c>
       <c r="O4" t="n">
-        <v>0.855</v>
+        <v>0.851</v>
       </c>
       <c r="P4" t="n">
-        <v>0.8179999999999999</v>
+        <v>0.819</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.785</v>
+        <v>0.784</v>
       </c>
       <c r="R4" t="n">
-        <v>0.726</v>
+        <v>0.724</v>
       </c>
       <c r="S4" t="n">
-        <v>0.614</v>
+        <v>0.611</v>
       </c>
       <c r="T4" t="n">
-        <v>0.488</v>
+        <v>0.48</v>
       </c>
       <c r="U4" t="n">
-        <v>0.25</v>
+        <v>0.242</v>
       </c>
       <c r="V4" t="n">
         <v>0.005</v>
@@ -2053,11 +2053,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>dino+u2net_sum</t>
+          <t>u2net+dino</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.9419419419419419</v>
       </c>
       <c r="C5" t="n">
         <v>0.9399999999999999</v>
@@ -2087,34 +2087,34 @@
         <v>0.907</v>
       </c>
       <c r="L5" t="n">
-        <v>0.889</v>
+        <v>0.891</v>
       </c>
       <c r="M5" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="N5" t="n">
         <v>0.877</v>
       </c>
-      <c r="N5" t="n">
-        <v>0.871</v>
-      </c>
       <c r="O5" t="n">
-        <v>0.847</v>
+        <v>0.855</v>
       </c>
       <c r="P5" t="n">
-        <v>0.8139999999999999</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.786</v>
+        <v>0.785</v>
       </c>
       <c r="R5" t="n">
-        <v>0.708</v>
+        <v>0.726</v>
       </c>
       <c r="S5" t="n">
-        <v>0.577</v>
+        <v>0.614</v>
       </c>
       <c r="T5" t="n">
-        <v>0.423</v>
+        <v>0.488</v>
       </c>
       <c r="U5" t="n">
-        <v>0.178</v>
+        <v>0.25</v>
       </c>
       <c r="V5" t="n">
         <v>0.005</v>
@@ -2127,7 +2127,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.9419419419419419</v>
       </c>
       <c r="C6" t="n">
         <v>0.9360000000000001</v>
@@ -2197,7 +2197,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.9419419419419419</v>
       </c>
       <c r="C7" t="n">
         <v>0.9360000000000001</v>
@@ -2267,7 +2267,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.9419419419419419</v>
       </c>
       <c r="C8" t="n">
         <v>0.9389999999999999</v>

</xml_diff>